<commit_message>
updated user histories for MVP
</commit_message>
<xml_diff>
--- a/Backlog_Seguimiento_Alternativa1_QUINOR.xlsx
+++ b/Backlog_Seguimiento_Alternativa1_QUINOR.xlsx
@@ -9,9 +9,10 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leyenda" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historias" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tec_Sprint1" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hallazgos" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tec_Sprint1" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hallazgos" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -717,7 +718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="22" customWidth="1" style="31" min="1" max="1"/>
@@ -888,41 +889,53 @@
       </c>
       <c r="B20" s="43" t="inlineStr">
         <is>
-          <t>Las 20 historias del backlog con dependencias, estado y bloqueos.</t>
+          <t>Las 14 historias del MVP con dependencias, estado y bloqueos.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="32">
       <c r="A21" s="42" t="inlineStr">
         <is>
-          <t>Resumen</t>
+          <t>Backlog</t>
         </is>
       </c>
       <c r="B21" s="43" t="inlineStr">
         <is>
-          <t>Puntos e historias por sprint y por estado. Todo calculado con formulas.</t>
+          <t>Las 6 historias postergadas fuera del MVP, con el motivo de cada una.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="32">
       <c r="A22" s="42" t="inlineStr">
         <is>
-          <t>Tec_Sprint1</t>
+          <t>Resumen</t>
         </is>
       </c>
       <c r="B22" s="43" t="inlineStr">
         <is>
-          <t>Verificacion de tecnologias necesarias para iniciar el Sprint 1.</t>
+          <t>Puntos e historias por sprint y por estado. Todo calculado con formulas.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="32">
       <c r="A23" s="42" t="inlineStr">
         <is>
+          <t>Tec_Sprint1</t>
+        </is>
+      </c>
+      <c r="B23" s="43" t="inlineStr">
+        <is>
+          <t>Verificacion de tecnologias necesarias para iniciar el Sprint 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="42" t="inlineStr">
+        <is>
           <t>Hallazgos</t>
         </is>
       </c>
-      <c r="B23" s="43" t="inlineStr">
+      <c r="B24" s="43" t="inlineStr">
         <is>
           <t>Inconsistencias detectadas en el documento funcional y su resolucion.</t>
         </is>
@@ -941,7 +954,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N25"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="31" min="1" max="1"/>
@@ -963,14 +976,14 @@
     <row r="1" ht="17.25" customHeight="1" s="32">
       <c r="A1" s="33" t="inlineStr">
         <is>
-          <t>Backlog de historias de usuario - Alternativa 1</t>
+          <t>Historias del MVP - Alternativa 1</t>
         </is>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="32">
       <c r="A2" s="34" t="inlineStr">
         <is>
-          <t>Columna Estado editable (NEW / PENDING / ACTIVE / DONE). Las demas se derivan del documento funcional.</t>
+          <t>MVP de 14 historias definido el 23/09/2026 (51 pts). Las 6 postergadas estan en la hoja Backlog. Columna Estado editable (NEW / PENDING / ACTIVE / DONE).</t>
         </is>
       </c>
     </row>
@@ -1220,7 +1233,7 @@
       </c>
       <c r="J7" s="47" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>HU-01 (S1), HU-02 (S1), HU-04 (S1)</t>
         </is>
       </c>
       <c r="K7" s="46" t="inlineStr">
@@ -1274,12 +1287,12 @@
       </c>
       <c r="H8" s="47" t="inlineStr">
         <is>
-          <t>HU-15</t>
+          <t>HU-14</t>
         </is>
       </c>
       <c r="I8" s="47" t="inlineStr">
         <is>
-          <t>HU-15 (S1)</t>
+          <t>HU-14 (S1)</t>
         </is>
       </c>
       <c r="J8" s="47" t="inlineStr">
@@ -1680,7 +1693,7 @@
       <c r="M14" s="47" t="n"/>
       <c r="N14" s="47" t="inlineStr">
         <is>
-          <t>Entregada el 18/09/2026, adelantada del Sprint 4. Su unica dependencia, HU-09, ya estaba DONE. CAMBIO DE ALCANCE acordado el 18/09/2026 y aplicado antes de desarrollar: esta historia queda solo con correo. Slack sale porque se esta evaluando Teams en su lugar, y el SMS sale con el: los dos son canales externos con proveedor, clave y costo por mensaje, y se evaluan juntos en una historia posterior. El criterio 1 se reescribio en consecuencia, aqui y en el documento funcional (apartados 2, 3, 5.2, 5.4 y 6.4). Los criterios 2 y 3 no cambian. DECISION IMPORTANTE: al quedarse las tres severidades en un solo canal, el criterio 1 se habria quedado sin contenido, porque las tres alertas serian el mismo correo, que es la forma mas rapida de que un supervisor deje de abrirlos. La severidad pasa a decidir a quien se avisa y con que urgencia: Alta a supervisores y administradores con asunto [ALERTA ALTA] y prioridad alta; Media y Baja solo a supervisores y con prioridad normal. El rol Consulta no recibe alertas de ningun nivel: es de solo lectura del dashboard y no le corresponde actuar sobre una carga. Los tres criterios verificados con 1220 pruebas automatizadas entre los cinco servicios (notificaciones 144, vlm 185, yolo 222, grabador 279, orquestador 390), 100% de cobertura en los cinco, y de punta a punta con MySQL, un buzon de correo real (mailpit) y el dashboard: el aviso salio 0,01 s despues del analisis, el correo llego a los dos supervisores y al administrador con X-Priority 1, la segunda vuelta del sondeo no mando un segundo correo, y los niveles Media y Baja salieron solo a supervisores y sin prioridad. Nuevo servicio quinor/despacho/notificaciones con POST /notificaciones (apartado 6.4, aiosmtplib). Va aparte por lo mismo que el de vision-lenguaje: es uno de los dos servicios que hablan con un servidor de fuera, y tenerlo aparte deja esa salida en un sitio que se puede cortar y vigilar. Los destinatarios salen de la tabla usuario de HU-15 y no de una lista en el entorno: dar de alta a alguien en el dashboard basta para que reciba alertas, y darlo de baja lo corta el mismo dia. Criterio 3: el reloj lo mide el grabador, que es el unico que sabe cuando quedo escrita la severidad, y el aviso sale en la misma pasada del analisis; esperar a la vuelta siguiente del sondeo gastaria media ventana sin hacer nada. El retraso real se guarda en notificacion.segundos_desde_analisis y se ve en el dashboard, de modo que el criterio se mide y no se supone. El correo no lleva fotogramas adjuntos: son imagenes de la zona de carga con personas dentro y el apartado 8 las quiere en la red interna; el enlace del criterio 2 lleva al dashboard, que pide sesion. Cambios de esquema: tabla notificacion, con clave unica (evento_id, canal) que impide el correo repetido en cada vuelta del sondeo. Un aviso fallido no cuenta como avisado y su fila se reemplaza en el siguiente intento: si contara, un relay caido un minuto dejaria un evento Alto sin correo para siempre. La columna canal se conserva aunque hoy solo valga 'correo', para que Teams o el SMS tengan su fila cuando entren. PENDIENTE: los datos del relay corporativo (host, puerto, credenciales y buzon de salida). Todo esta probado contra mailpit y contra un servidor SMTP real levantado en las pruebas; el primer correo de verdad espera a que QUINOR provea esos datos. Ver README de quinor/despacho/notificaciones.</t>
+          <t>Entregada el 18/09/2026, adelantada del Sprint 4. Su unica dependencia, HU-09, ya estaba DONE. CAMBIO DE ALCANCE acordado el 18/09/2026 y aplicado antes de desarrollar: esta historia queda solo con correo. Slack sale porque se esta evaluando Teams en su lugar, y el SMS sale con el: los dos son canales externos con proveedor, clave y costo por mensaje, y se evaluan juntos en una historia posterior. El criterio 1 se reescribio en consecuencia, aqui y en el documento funcional (apartados 2, 3, 5.2, 5.4 y 6.4). Los criterios 2 y 3 no cambian. DECISION IMPORTANTE: al quedarse las tres severidades en un solo canal, el criterio 1 se habria quedado sin contenido, porque las tres alertas serian el mismo correo, que es la forma mas rapida de que un supervisor deje de abrirlos. La severidad pasa a decidir a quien se avisa y con que urgencia: Alta a supervisores y administradores con asunto [ALERTA ALTA] y prioridad alta; Media y Baja solo a supervisores y con prioridad normal. El rol Consulta no recibe alertas de ningun nivel: es de solo lectura del dashboard y no le corresponde actuar sobre una carga. Los tres criterios verificados con 1220 pruebas automatizadas entre los cinco servicios (notificaciones 144, vlm 185, yolo 222, grabador 279, orquestador 390), 100% de cobertura en los cinco, y de punta a punta con MySQL, un buzon de correo real (mailpit) y el dashboard: el aviso salio 0,01 s despues del analisis, el correo llego a los dos supervisores y al administrador con X-Priority 1, la segunda vuelta del sondeo no mando un segundo correo, y los niveles Media y Baja salieron solo a supervisores y sin prioridad. Nuevo servicio quinor/despacho/notificaciones con POST /notificaciones (apartado 6.4, aiosmtplib). Va aparte por lo mismo que el de vision-lenguaje: es uno de los dos servicios que hablan con un servidor de fuera, y tenerlo aparte deja esa salida en un sitio que se puede cortar y vigilar. Los destinatarios salen de la tabla usuario de HU-14 y no de una lista en el entorno: dar de alta a alguien en el dashboard basta para que reciba alertas, y darlo de baja lo corta el mismo dia. Criterio 3: el reloj lo mide el grabador, que es el unico que sabe cuando quedo escrita la severidad, y el aviso sale en la misma pasada del analisis; esperar a la vuelta siguiente del sondeo gastaria media ventana sin hacer nada. El retraso real se guarda en notificacion.segundos_desde_analisis y se ve en el dashboard, de modo que el criterio se mide y no se supone. El correo no lleva fotogramas adjuntos: son imagenes de la zona de carga con personas dentro y el apartado 8 las quiere en la red interna; el enlace del criterio 2 lleva al dashboard, que pide sesion. Cambios de esquema: tabla notificacion, con clave unica (evento_id, canal) que impide el correo repetido en cada vuelta del sondeo. Un aviso fallido no cuenta como avisado y su fila se reemplaza en el siguiente intento: si contara, un relay caido un minuto dejaria un evento Alto sin correo para siempre. La columna canal se conserva aunque hoy solo valga 'correo', para que Teams o el SMS tengan su fila cuando entren. PENDIENTE: los datos del relay corporativo (host, puerto, credenciales y buzon de salida). Todo esta probado contra mailpit y contra un servidor SMTP real levantado en las pruebas; el primer correo de verdad espera a que QUINOR provea esos datos. Ver README de quinor/despacho/notificaciones.</t>
         </is>
       </c>
     </row>
@@ -1755,7 +1768,7 @@
         </is>
       </c>
       <c r="B16" s="46" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C16" s="47" t="inlineStr">
         <is>
@@ -1794,7 +1807,7 @@
       </c>
       <c r="J16" s="47" t="inlineStr">
         <is>
-          <t>HU-06 (S2), HU-09 (S4), HU-11 (S2)</t>
+          <t>HU-06 (S2), HU-11 (S2)</t>
         </is>
       </c>
       <c r="K16" s="46" t="inlineStr">
@@ -1808,7 +1821,7 @@
       <c r="M16" s="47" t="n"/>
       <c r="N16" s="47" t="inlineStr">
         <is>
-          <t>Sus dependencias HU-06, HU-07, HU-08 y, desde el 17/09/2026, HU-09 estan DONE: el detalle ya muestra pesos, conteo, personas, descripcion y severidad, y los fotogramas clave ya se guardan en MinIO con su motivo y su segundo, que es el criterio 3. Falta HU-11 para la lista y reproducir el clip en el navegador, que es lo propio de esta historia.</t>
+          <t>Sus dependencias HU-06, HU-07, HU-08 y, desde el 17/09/2026, HU-09 estan DONE: el detalle ya muestra pesos, conteo, personas, descripcion y severidad, y los fotogramas clave ya se guardan en MinIO con su motivo y su segundo, que es el criterio 3. Falta HU-11 para la lista y reproducir el clip en el navegador, que es lo propio de esta historia. 23/09/2026: movida del Sprint 3 al Sprint 4 al definir el MVP, porque depende de HU-09 (Sprint 4) y no puede ir en un sprint anterior a su dependencia.</t>
         </is>
       </c>
     </row>
@@ -1819,7 +1832,7 @@
         </is>
       </c>
       <c r="B17" s="46" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C17" s="47" t="inlineStr">
         <is>
@@ -1848,17 +1861,17 @@
       </c>
       <c r="H17" s="47" t="inlineStr">
         <is>
-          <t>HU-12, HU-15</t>
+          <t>HU-12, HU-14</t>
         </is>
       </c>
       <c r="I17" s="47" t="inlineStr">
         <is>
-          <t>HU-12 (S3), HU-15 (S1)</t>
+          <t>HU-12 (S4), HU-14 (S1)</t>
         </is>
       </c>
       <c r="J17" s="47" t="inlineStr">
         <is>
-          <t>HU-15 (S1)</t>
+          <t>HU-14 (S1)</t>
         </is>
       </c>
       <c r="K17" s="46" t="inlineStr">
@@ -1872,7 +1885,7 @@
       <c r="M17" s="47" t="n"/>
       <c r="N17" s="47" t="inlineStr">
         <is>
-          <t>Excluida del conteo del sprint: depende de historias de otro sprint.</t>
+          <t>Excluida del conteo del sprint: depende de historias de otro sprint. 23/09/2026: movida del Sprint 3 al Sprint 4 junto con HU-12, de la que depende.</t>
         </is>
       </c>
     </row>
@@ -1883,83 +1896,19 @@
         </is>
       </c>
       <c r="B18" s="46" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C18" s="47" t="inlineStr">
         <is>
-          <t>Reportes</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="D18" s="47" t="inlineStr">
         <is>
-          <t>Como gerente de operaciones, quiero generar un reporte semanal de discrepancias con totales por severidad, turno y estado, para medir la tendencia de perdidas y falsos positivos.</t>
+          <t>Como administrador del sistema, quiero gestionar usuarios y roles (Administrador, Supervisor, Consulta), para que cada persona solo acceda a lo que le corresponde.</t>
         </is>
       </c>
       <c r="E18" s="47" t="inlineStr">
-        <is>
-          <t>1. El reporte se genera en PDF y Excel desde el dashboard.
-2. Incluye tabla resumen y grafico de eventos por dia.
-3. Se puede elegir cualquier rango de fechas.</t>
-        </is>
-      </c>
-      <c r="F18" s="46" t="inlineStr">
-        <is>
-          <t>Should</t>
-        </is>
-      </c>
-      <c r="G18" s="46" t="n">
-        <v>3</v>
-      </c>
-      <c r="H18" s="47" t="inlineStr">
-        <is>
-          <t>HU-11</t>
-        </is>
-      </c>
-      <c r="I18" s="47" t="inlineStr">
-        <is>
-          <t>HU-11 (S2)</t>
-        </is>
-      </c>
-      <c r="J18" s="47" t="inlineStr">
-        <is>
-          <t>HU-11 (S2)</t>
-        </is>
-      </c>
-      <c r="K18" s="46" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="L18" s="48" t="n">
-        <v>0</v>
-      </c>
-      <c r="M18" s="47" t="n"/>
-      <c r="N18" s="47" t="inlineStr">
-        <is>
-          <t>Excluida del conteo del sprint: depende de historias de otro sprint.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="73.5" customHeight="1" s="32">
-      <c r="A19" s="45" t="inlineStr">
-        <is>
-          <t>HU-15</t>
-        </is>
-      </c>
-      <c r="B19" s="46" t="n">
-        <v>1</v>
-      </c>
-      <c r="C19" s="47" t="inlineStr">
-        <is>
-          <t>Seguridad</t>
-        </is>
-      </c>
-      <c r="D19" s="47" t="inlineStr">
-        <is>
-          <t>Como administrador del sistema, quiero gestionar usuarios y roles (Administrador, Supervisor, Consulta), para que cada persona solo acceda a lo que le corresponde.</t>
-        </is>
-      </c>
-      <c r="E19" s="47" t="inlineStr">
         <is>
           <t>1. Se pueden crear, desactivar y asignar roles a usuarios.
 2. El rol Consulta no puede cambiar estados ni configuraciones.
@@ -1967,408 +1916,93 @@
 4. La autenticacion usa token opaco en tabla api_token, revocable desde el dashboard.</t>
         </is>
       </c>
-      <c r="F19" s="46" t="inlineStr">
+      <c r="F18" s="46" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="G19" s="46" t="n">
+      <c r="G18" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="H19" s="47" t="inlineStr">
+      <c r="H18" s="47" t="inlineStr">
         <is>
           <t>Ninguna</t>
         </is>
       </c>
-      <c r="I19" s="47" t="inlineStr">
+      <c r="I18" s="47" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="J19" s="47" t="inlineStr">
+      <c r="J18" s="47" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="K19" s="46" t="inlineStr">
+      <c r="K18" s="46" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
       </c>
-      <c r="L19" s="48" t="n">
+      <c r="L18" s="48" t="n">
         <v>1</v>
       </c>
-      <c r="M19" s="47" t="n"/>
-      <c r="N19" s="47" t="inlineStr">
-        <is>
-          <t>Entregada el 14/09/2026. Los cuatro criterios verificados con 214 pruebas automatizadas y 100% de cobertura. Autenticacion por token opaco en la tabla api_token, con revocacion inmediata desde el dashboard. Ver README, apartado HU-15.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="73.5" customHeight="1" s="32">
-      <c r="A20" s="45" t="inlineStr">
-        <is>
-          <t>HU-16</t>
-        </is>
-      </c>
-      <c r="B20" s="46" t="n">
-        <v>4</v>
-      </c>
-      <c r="C20" s="47" t="inlineStr">
-        <is>
-          <t>Seguridad</t>
-        </is>
-      </c>
-      <c r="D20" s="47" t="inlineStr">
-        <is>
-          <t>Como auditor interno, quiero consultar el historial de acciones realizadas sobre cada evento, para contar con evidencia trazable ante una investigacion de personal.</t>
-        </is>
-      </c>
-      <c r="E20" s="47" t="inlineStr">
-        <is>
-          <t>1. Cada cambio de estado, comentario o configuracion queda en una tabla de auditoria inmutable.
-2. El historial es visible en el detalle del evento.
-3. Los registros de auditoria no pueden borrarse desde la aplicacion.</t>
-        </is>
-      </c>
-      <c r="F20" s="46" t="inlineStr">
-        <is>
-          <t>Should</t>
-        </is>
-      </c>
-      <c r="G20" s="46" t="n">
-        <v>2</v>
-      </c>
-      <c r="H20" s="47" t="inlineStr">
-        <is>
-          <t>HU-13</t>
-        </is>
-      </c>
-      <c r="I20" s="47" t="inlineStr">
-        <is>
-          <t>HU-13 (S3)</t>
-        </is>
-      </c>
-      <c r="J20" s="47" t="inlineStr">
-        <is>
-          <t>HU-13 (S3)</t>
-        </is>
-      </c>
-      <c r="K20" s="46" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="L20" s="48" t="n">
-        <v>0</v>
-      </c>
-      <c r="M20" s="47" t="n"/>
-      <c r="N20" s="47" t="inlineStr">
-        <is>
-          <t>Excluida del conteo del sprint: depende de historias de otro sprint.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="73.5" customHeight="1" s="32">
-      <c r="A21" s="45" t="inlineStr">
-        <is>
-          <t>HU-17</t>
-        </is>
-      </c>
-      <c r="B21" s="46" t="n">
-        <v>1</v>
-      </c>
-      <c r="C21" s="47" t="inlineStr">
-        <is>
-          <t>Plataforma</t>
-        </is>
-      </c>
-      <c r="D21" s="47" t="inlineStr">
-        <is>
-          <t>Como administrador del sistema, quiero que el analisis de video se procese en cola con reintentos automaticos, para que una falla temporal no deje eventos sin analizar.</t>
-        </is>
-      </c>
-      <c r="E21" s="47" t="inlineStr">
-        <is>
-          <t>1. Cada analisis es una tarea Celery con hasta 3 reintentos y espera exponencial.
-2. Las tareas fallidas quedan visibles en el panel de salud.
-3. El orquestador nunca bloquea el registro de pesadas mientras analiza video.</t>
-        </is>
-      </c>
-      <c r="F21" s="46" t="inlineStr">
-        <is>
-          <t>Must</t>
-        </is>
-      </c>
-      <c r="G21" s="46" t="n">
-        <v>3</v>
-      </c>
-      <c r="H21" s="47" t="inlineStr">
-        <is>
-          <t>HU-03</t>
-        </is>
-      </c>
-      <c r="I21" s="47" t="inlineStr">
-        <is>
-          <t>HU-03 (S2)</t>
-        </is>
-      </c>
-      <c r="J21" s="47" t="inlineStr">
-        <is>
-          <t>HU-03 (S2)</t>
-        </is>
-      </c>
-      <c r="K21" s="46" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="L21" s="48" t="n">
-        <v>0</v>
-      </c>
-      <c r="M21" s="47" t="n"/>
-      <c r="N21" s="47" t="inlineStr">
-        <is>
-          <t>Excluida del conteo del sprint: dependia de HU-03, del Sprint 2. Al 14/09/2026 esa dependencia esta DONE, asi que HU-17 ya no esta bloqueada y se puede planificar. Cambiar su estado a NEW es una decision de planificacion: subiria los puntos computables del Sprint 1 de 11 a 14.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="73.5" customHeight="1" s="32">
-      <c r="A22" s="45" t="inlineStr">
-        <is>
-          <t>HU-18</t>
-        </is>
-      </c>
-      <c r="B22" s="46" t="n">
-        <v>5</v>
-      </c>
-      <c r="C22" s="47" t="inlineStr">
-        <is>
-          <t>Plataforma</t>
-        </is>
-      </c>
-      <c r="D22" s="47" t="inlineStr">
-        <is>
-          <t>Como administrador del sistema, quiero ver un panel de salud con el estado de bascula, camaras, cola de tareas y servicios de IA, para detectar fallas del sistema antes de que se pierdan eventos.</t>
-        </is>
-      </c>
-      <c r="E22" s="47" t="inlineStr">
-        <is>
-          <t>1. Cada componente muestra estado OK, Advertencia o Error y ultima verificacion.
-2. Un componente en Error genera una alerta al administrador.
-3. El panel se actualiza cada 30 s.</t>
-        </is>
-      </c>
-      <c r="F22" s="46" t="inlineStr">
-        <is>
-          <t>Should</t>
-        </is>
-      </c>
-      <c r="G22" s="46" t="n">
-        <v>3</v>
-      </c>
-      <c r="H22" s="47" t="inlineStr">
-        <is>
-          <t>HU-01, HU-05, HU-17</t>
-        </is>
-      </c>
-      <c r="I22" s="47" t="inlineStr">
-        <is>
-          <t>HU-01 (S1), HU-05 (S2), HU-17 (S1)</t>
-        </is>
-      </c>
-      <c r="J22" s="47" t="inlineStr">
-        <is>
-          <t>HU-01 (S1), HU-05 (S2), HU-17 (S1)</t>
-        </is>
-      </c>
-      <c r="K22" s="46" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="L22" s="48" t="n">
-        <v>0</v>
-      </c>
-      <c r="M22" s="47" t="n"/>
-      <c r="N22" s="47" t="inlineStr">
-        <is>
-          <t>Excluida del conteo del sprint: depende de historias de otro sprint.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="73.5" customHeight="1" s="32">
-      <c r="A23" s="45" t="inlineStr">
-        <is>
-          <t>HU-19</t>
-        </is>
-      </c>
-      <c r="B23" s="46" t="n">
-        <v>5</v>
-      </c>
-      <c r="C23" s="47" t="inlineStr">
-        <is>
-          <t>Analisis IA</t>
-        </is>
-      </c>
-      <c r="D23" s="47" t="inlineStr">
-        <is>
-          <t>Como ingeniero de datos, quiero reentrenar el modelo YOLO con imagenes etiquetadas de sacos de quinua de la planta, para mejorar la precision del conteo con datos propios.</t>
-        </is>
-      </c>
-      <c r="E23" s="47" t="inlineStr">
-        <is>
-          <t>1. Existe un script que toma un dataset en formato YOLO y entrena un nuevo modelo.
-2. El nuevo modelo solo se despliega si supera la precision del anterior en el set de validacion.
-3. Se conserva el historial de versiones del modelo.</t>
-        </is>
-      </c>
-      <c r="F23" s="46" t="inlineStr">
-        <is>
-          <t>Should</t>
-        </is>
-      </c>
-      <c r="G23" s="46" t="n">
-        <v>5</v>
-      </c>
-      <c r="H23" s="47" t="inlineStr">
-        <is>
-          <t>HU-07</t>
-        </is>
-      </c>
-      <c r="I23" s="47" t="inlineStr">
-        <is>
-          <t>HU-07 (S3)</t>
-        </is>
-      </c>
-      <c r="J23" s="47" t="inlineStr">
-        <is>
-          <t>HU-07 (S3)</t>
-        </is>
-      </c>
-      <c r="K23" s="46" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="L23" s="48" t="n">
-        <v>0</v>
-      </c>
-      <c r="M23" s="47" t="n"/>
-      <c r="N23" s="47" t="inlineStr">
-        <is>
-          <t>Desbloqueada el 16/09/2026: HU-07, su unica dependencia, esta DONE. Es ademas la que sustituye el set sintetico de validacion por el dataset real etiquetado de la rampa y versiona el modelo en la tabla modelo_version; mientras tanto el nombre del archivo de pesos hace de version y viaja en cada respuesta del servicio.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="73.5" customHeight="1" s="32">
-      <c r="A24" s="45" t="inlineStr">
-        <is>
-          <t>HU-20</t>
-        </is>
-      </c>
-      <c r="B24" s="46" t="n">
-        <v>5</v>
-      </c>
-      <c r="C24" s="47" t="inlineStr">
-        <is>
-          <t>Reportes</t>
-        </is>
-      </c>
-      <c r="D24" s="47" t="inlineStr">
-        <is>
-          <t>Como gerente de operaciones, quiero exportar la lista de eventos filtrada a CSV, para analizar la informacion en otras herramientas.</t>
-        </is>
-      </c>
-      <c r="E24" s="47" t="inlineStr">
-        <is>
-          <t>1. El boton Exportar respeta los filtros activos.
-2. El archivo incluye todas las columnas del evento y su estado.
-3. La exportacion de hasta 10 000 eventos tarda menos de 10 s.</t>
-        </is>
-      </c>
-      <c r="F24" s="46" t="inlineStr">
-        <is>
-          <t>Could</t>
-        </is>
-      </c>
-      <c r="G24" s="46" t="n">
-        <v>1</v>
-      </c>
-      <c r="H24" s="47" t="inlineStr">
-        <is>
-          <t>HU-11</t>
-        </is>
-      </c>
-      <c r="I24" s="47" t="inlineStr">
-        <is>
-          <t>HU-11 (S2)</t>
-        </is>
-      </c>
-      <c r="J24" s="47" t="inlineStr">
-        <is>
-          <t>HU-11 (S2)</t>
-        </is>
-      </c>
-      <c r="K24" s="46" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="L24" s="48" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" s="47" t="n"/>
-      <c r="N24" s="47" t="inlineStr">
-        <is>
-          <t>Excluida del conteo del sprint: depende de historias de otro sprint.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="15" customHeight="1" s="32">
-      <c r="A25" s="49" t="inlineStr">
+      <c r="M18" s="47" t="n"/>
+      <c r="N18" s="47" t="inlineStr">
+        <is>
+          <t>Entregada el 14/09/2026. Los cuatro criterios verificados con 214 pruebas automatizadas y 100% de cobertura. Autenticacion por token opaco en la tabla api_token, con revocacion inmediata desde el dashboard. Ver README, apartado HU-14. 23/09/2026: renumerada desde HU-15 al definir el MVP de 14 historias. El codigo y los README aun la citan como HU-15.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1" s="32">
+      <c r="A19" s="49" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B25" s="50" t="n"/>
-      <c r="C25" s="50" t="n"/>
-      <c r="D25" s="50" t="n"/>
-      <c r="E25" s="50" t="n"/>
-      <c r="F25" s="50" t="n"/>
-      <c r="G25" s="51">
-        <f>SUM(G5:G24)</f>
-        <v/>
-      </c>
-      <c r="H25" s="50" t="n"/>
-      <c r="I25" s="50" t="n"/>
-      <c r="J25" s="50" t="n"/>
-      <c r="K25" s="50" t="n"/>
-      <c r="L25" s="50" t="n"/>
-      <c r="M25" s="50" t="n"/>
-      <c r="N25" s="50" t="n"/>
-    </row>
+      <c r="B19" s="50" t="n"/>
+      <c r="C19" s="50" t="n"/>
+      <c r="D19" s="50" t="n"/>
+      <c r="E19" s="50" t="n"/>
+      <c r="F19" s="50" t="n"/>
+      <c r="G19" s="51">
+        <f>SUM(G5:G18)</f>
+        <v/>
+      </c>
+      <c r="H19" s="50" t="n"/>
+      <c r="I19" s="50" t="n"/>
+      <c r="J19" s="50" t="n"/>
+      <c r="K19" s="50" t="n"/>
+      <c r="L19" s="50" t="n"/>
+      <c r="M19" s="50" t="n"/>
+      <c r="N19" s="50" t="n"/>
+    </row>
+    <row r="20" s="32"/>
+    <row r="21" s="32"/>
+    <row r="22" s="32"/>
+    <row r="23" s="32"/>
+    <row r="24" s="32"/>
+    <row r="25" s="32"/>
   </sheetData>
-  <conditionalFormatting sqref="K5:K24">
-    <cfRule type="cellIs" rank="0" priority="2" equalAverage="0" operator="equal" aboveAverage="0" dxfId="0" text="" percent="0" bottom="0">
+  <conditionalFormatting sqref="K5:K18">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"NEW"</formula>
     </cfRule>
-    <cfRule type="cellIs" rank="0" priority="3" equalAverage="0" operator="equal" aboveAverage="0" dxfId="1" text="" percent="0" bottom="0">
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
       <formula>"PENDING"</formula>
     </cfRule>
-    <cfRule type="cellIs" rank="0" priority="4" equalAverage="0" operator="equal" aboveAverage="0" dxfId="2" text="" percent="0" bottom="0">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
       <formula>"ACTIVE"</formula>
     </cfRule>
-    <cfRule type="cellIs" rank="0" priority="5" equalAverage="0" operator="equal" aboveAverage="0" dxfId="3" text="" percent="0" bottom="0">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
       <formula>"DONE"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="K5:K24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Estado invalido" error="Solo se admite NEW, PENDING, ACTIVE o DONE." type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="K5:K18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"NEW,PENDING,ACTIVE,DONE"</formula1>
-      <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="L5:L24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="decimal" errorStyle="stop" operator="between">
+    <dataValidation sqref="L5:L18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="decimal" operator="between">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
@@ -2385,7 +2019,607 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:O11"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="9" customWidth="1" style="31" min="1" max="1"/>
+    <col width="7" customWidth="1" style="31" min="2" max="2"/>
+    <col width="17" customWidth="1" style="31" min="3" max="3"/>
+    <col width="64" customWidth="1" style="31" min="4" max="4"/>
+    <col width="62" customWidth="1" style="31" min="5" max="5"/>
+    <col width="7" customWidth="1" style="31" min="6" max="6"/>
+    <col width="6" customWidth="1" style="31" min="7" max="7"/>
+    <col width="16" customWidth="1" style="31" min="8" max="8"/>
+    <col width="24" customWidth="1" style="31" min="9" max="9"/>
+    <col width="22" customWidth="1" style="31" min="10" max="10"/>
+    <col width="11" customWidth="1" style="31" min="11" max="11"/>
+    <col width="10" customWidth="1" style="31" min="12" max="12"/>
+    <col width="16" customWidth="1" style="31" min="13" max="13"/>
+    <col width="40" customWidth="1" style="31" min="14" max="14"/>
+    <col width="40" customWidth="1" style="32" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="17.25" customHeight="1" s="32">
+      <c r="A1" s="33" t="inlineStr">
+        <is>
+          <t>Backlog post-MVP - historias postergadas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1" s="32">
+      <c r="A2" s="34" t="inlineStr">
+        <is>
+          <t>6 historias (17 pts) que quedan fuera del MVP definido el 23/09/2026. Columna Estado editable. La columna O explica por que se posterga cada una.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4" ht="23.25" customHeight="1" s="32">
+      <c r="A4" s="44" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B4" s="44" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="C4" s="44" t="inlineStr">
+        <is>
+          <t>Categoria</t>
+        </is>
+      </c>
+      <c r="D4" s="44" t="inlineStr">
+        <is>
+          <t>Historia de usuario</t>
+        </is>
+      </c>
+      <c r="E4" s="44" t="inlineStr">
+        <is>
+          <t>Criterios de aceptacion</t>
+        </is>
+      </c>
+      <c r="F4" s="44" t="inlineStr">
+        <is>
+          <t>Prio.</t>
+        </is>
+      </c>
+      <c r="G4" s="44" t="inlineStr">
+        <is>
+          <t>Pts.</t>
+        </is>
+      </c>
+      <c r="H4" s="44" t="inlineStr">
+        <is>
+          <t>Depende de</t>
+        </is>
+      </c>
+      <c r="I4" s="44" t="inlineStr">
+        <is>
+          <t>Sprint de cada dependencia</t>
+        </is>
+      </c>
+      <c r="J4" s="44" t="inlineStr">
+        <is>
+          <t>Dependencia cruzada</t>
+        </is>
+      </c>
+      <c r="K4" s="44" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="L4" s="44" t="inlineStr">
+        <is>
+          <t>Avance %</t>
+        </is>
+      </c>
+      <c r="M4" s="44" t="inlineStr">
+        <is>
+          <t>Responsable</t>
+        </is>
+      </c>
+      <c r="N4" s="44" t="inlineStr">
+        <is>
+          <t>Observaciones</t>
+        </is>
+      </c>
+      <c r="O4" s="44" t="inlineStr">
+        <is>
+          <t>Motivo de postergacion</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="73.5" customHeight="1" s="32">
+      <c r="A5" s="45" t="inlineStr">
+        <is>
+          <t>HU-15</t>
+        </is>
+      </c>
+      <c r="B5" s="46" t="n">
+        <v>5</v>
+      </c>
+      <c r="C5" s="47" t="inlineStr">
+        <is>
+          <t>Reportes</t>
+        </is>
+      </c>
+      <c r="D5" s="47" t="inlineStr">
+        <is>
+          <t>Como gerente de operaciones, quiero generar un reporte semanal de discrepancias con totales por severidad, turno y estado, para medir la tendencia de perdidas y falsos positivos.</t>
+        </is>
+      </c>
+      <c r="E5" s="47" t="inlineStr">
+        <is>
+          <t>1. El reporte se genera en PDF y Excel desde el dashboard.
+2. Incluye tabla resumen y grafico de eventos por dia.
+3. Se puede elegir cualquier rango de fechas.</t>
+        </is>
+      </c>
+      <c r="F5" s="46" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G5" s="46" t="n">
+        <v>3</v>
+      </c>
+      <c r="H5" s="47" t="inlineStr">
+        <is>
+          <t>HU-11</t>
+        </is>
+      </c>
+      <c r="I5" s="47" t="inlineStr">
+        <is>
+          <t>HU-11 (S2)</t>
+        </is>
+      </c>
+      <c r="J5" s="47" t="inlineStr">
+        <is>
+          <t>HU-11 (S2)</t>
+        </is>
+      </c>
+      <c r="K5" s="46" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="L5" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="47" t="n"/>
+      <c r="N5" s="47" t="inlineStr">
+        <is>
+          <t>Postergada fuera del MVP el 23/09/2026. Renumerada desde HU-14 para que la hoja Historias quede sin huecos. Excluida del conteo del sprint: depende de historias de otro sprint.</t>
+        </is>
+      </c>
+      <c r="O5" s="47" t="inlineStr">
+        <is>
+          <t>Mide tendencias de varias semanas; no hace falta para validar el MVP ni para actuar antes de que salga el contenedor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="73.5" customHeight="1" s="32">
+      <c r="A6" s="45" t="inlineStr">
+        <is>
+          <t>HU-16</t>
+        </is>
+      </c>
+      <c r="B6" s="46" t="n">
+        <v>4</v>
+      </c>
+      <c r="C6" s="47" t="inlineStr">
+        <is>
+          <t>Seguridad</t>
+        </is>
+      </c>
+      <c r="D6" s="47" t="inlineStr">
+        <is>
+          <t>Como auditor interno, quiero consultar el historial de acciones realizadas sobre cada evento, para contar con evidencia trazable ante una investigacion de personal.</t>
+        </is>
+      </c>
+      <c r="E6" s="47" t="inlineStr">
+        <is>
+          <t>1. Cada cambio de estado, comentario o configuracion queda en una tabla de auditoria inmutable.
+2. El historial es visible en el detalle del evento.
+3. Los registros de auditoria no pueden borrarse desde la aplicacion.</t>
+        </is>
+      </c>
+      <c r="F6" s="46" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G6" s="46" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" s="47" t="inlineStr">
+        <is>
+          <t>HU-13</t>
+        </is>
+      </c>
+      <c r="I6" s="47" t="inlineStr">
+        <is>
+          <t>HU-13 (S4)</t>
+        </is>
+      </c>
+      <c r="J6" s="47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K6" s="46" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="L6" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="47" t="n"/>
+      <c r="N6" s="47" t="inlineStr">
+        <is>
+          <t>Excluida del conteo del sprint: depende de historias de otro sprint. 23/09/2026: HU-13 paso al Sprint 4, asi que la dependencia deja de ser cruzada.</t>
+        </is>
+      </c>
+      <c r="O6" s="47" t="inlineStr">
+        <is>
+          <t>Los criterios 1 y 3 ya los garantiza el motor (tabla auditoria y triggers trg_auditoria_no_update / no_delete). Solo falta mostrar el historial, que no afecta a ningun indicador del piloto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="73.5" customHeight="1" s="32">
+      <c r="A7" s="45" t="inlineStr">
+        <is>
+          <t>HU-17</t>
+        </is>
+      </c>
+      <c r="B7" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="47" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="D7" s="47" t="inlineStr">
+        <is>
+          <t>Como administrador del sistema, quiero que el analisis de video se procese en cola con reintentos automaticos, para que una falla temporal no deje eventos sin analizar.</t>
+        </is>
+      </c>
+      <c r="E7" s="47" t="inlineStr">
+        <is>
+          <t>1. Cada analisis es una tarea Celery con hasta 3 reintentos y espera exponencial.
+2. Las tareas fallidas quedan visibles en el panel de salud.
+3. El orquestador nunca bloquea el registro de pesadas mientras analiza video.</t>
+        </is>
+      </c>
+      <c r="F7" s="46" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G7" s="46" t="n">
+        <v>3</v>
+      </c>
+      <c r="H7" s="47" t="inlineStr">
+        <is>
+          <t>HU-03</t>
+        </is>
+      </c>
+      <c r="I7" s="47" t="inlineStr">
+        <is>
+          <t>HU-03 (S2)</t>
+        </is>
+      </c>
+      <c r="J7" s="47" t="inlineStr">
+        <is>
+          <t>HU-03 (S2)</t>
+        </is>
+      </c>
+      <c r="K7" s="46" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="L7" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="47" t="n"/>
+      <c r="N7" s="47" t="inlineStr">
+        <is>
+          <t>Excluida del conteo del sprint: dependia de HU-03, del Sprint 2. Al 14/09/2026 esa dependencia esta DONE, asi que HU-17 ya no esta bloqueada y se puede planificar. Cambiar su estado a NEW es una decision de planificacion: subiria los puntos computables del Sprint 1 de 11 a 14.</t>
+        </is>
+      </c>
+      <c r="O7" s="47" t="inlineStr">
+        <is>
+          <t>El bucle del grabador ya hace de worker con su pasada de reintentos y el criterio 3 se cumple por estar en otro proceso. Su criterio 2 depende de HU-18. Queda PENDING por decision del usuario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="73.5" customHeight="1" s="32">
+      <c r="A8" s="45" t="inlineStr">
+        <is>
+          <t>HU-18</t>
+        </is>
+      </c>
+      <c r="B8" s="46" t="n">
+        <v>5</v>
+      </c>
+      <c r="C8" s="47" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="D8" s="47" t="inlineStr">
+        <is>
+          <t>Como administrador del sistema, quiero ver un panel de salud con el estado de bascula, camaras, cola de tareas y servicios de IA, para detectar fallas del sistema antes de que se pierdan eventos.</t>
+        </is>
+      </c>
+      <c r="E8" s="47" t="inlineStr">
+        <is>
+          <t>1. Cada componente muestra estado OK, Advertencia o Error y ultima verificacion.
+2. Un componente en Error genera una alerta al administrador.
+3. El panel se actualiza cada 30 s.</t>
+        </is>
+      </c>
+      <c r="F8" s="46" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G8" s="46" t="n">
+        <v>3</v>
+      </c>
+      <c r="H8" s="47" t="inlineStr">
+        <is>
+          <t>HU-01, HU-05, HU-17</t>
+        </is>
+      </c>
+      <c r="I8" s="47" t="inlineStr">
+        <is>
+          <t>HU-01 (S1), HU-05 (S2), HU-17 (S1)</t>
+        </is>
+      </c>
+      <c r="J8" s="47" t="inlineStr">
+        <is>
+          <t>HU-01 (S1), HU-05 (S2), HU-17 (S1)</t>
+        </is>
+      </c>
+      <c r="K8" s="46" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="L8" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="47" t="n"/>
+      <c r="N8" s="47" t="inlineStr">
+        <is>
+          <t>Excluida del conteo del sprint: depende de historias de otro sprint.</t>
+        </is>
+      </c>
+      <c r="O8" s="47" t="inlineStr">
+        <is>
+          <t>Depende de HU-17. Mientras tanto salud_componente y GET /salud registran los fallos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="73.5" customHeight="1" s="32">
+      <c r="A9" s="45" t="inlineStr">
+        <is>
+          <t>HU-19</t>
+        </is>
+      </c>
+      <c r="B9" s="46" t="n">
+        <v>5</v>
+      </c>
+      <c r="C9" s="47" t="inlineStr">
+        <is>
+          <t>Analisis IA</t>
+        </is>
+      </c>
+      <c r="D9" s="47" t="inlineStr">
+        <is>
+          <t>Como ingeniero de datos, quiero reentrenar el modelo YOLO con imagenes etiquetadas de sacos de quinua de la planta, para mejorar la precision del conteo con datos propios.</t>
+        </is>
+      </c>
+      <c r="E9" s="47" t="inlineStr">
+        <is>
+          <t>1. Existe un script que toma un dataset en formato YOLO y entrena un nuevo modelo.
+2. El nuevo modelo solo se despliega si supera la precision del anterior en el set de validacion.
+3. Se conserva el historial de versiones del modelo.</t>
+        </is>
+      </c>
+      <c r="F9" s="46" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G9" s="46" t="n">
+        <v>5</v>
+      </c>
+      <c r="H9" s="47" t="inlineStr">
+        <is>
+          <t>HU-07</t>
+        </is>
+      </c>
+      <c r="I9" s="47" t="inlineStr">
+        <is>
+          <t>HU-07 (S3)</t>
+        </is>
+      </c>
+      <c r="J9" s="47" t="inlineStr">
+        <is>
+          <t>HU-07 (S3)</t>
+        </is>
+      </c>
+      <c r="K9" s="46" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="L9" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="47" t="n"/>
+      <c r="N9" s="47" t="inlineStr">
+        <is>
+          <t>Desbloqueada el 16/09/2026: HU-07, su unica dependencia, esta DONE. Es ademas la que sustituye el set sintetico de validacion por el dataset real etiquetado de la rampa y versiona el modelo en la tabla modelo_version; mientras tanto el nombre del archivo de pesos hace de version y viaja en cada respuesta del servicio.</t>
+        </is>
+      </c>
+      <c r="O9" s="47" t="inlineStr">
+        <is>
+          <t>Requiere el dataset real de sacos de yute que debe aportar QUINOR. Encaja despues del piloto, cuando haya imagenes de planta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="73.5" customHeight="1" s="32">
+      <c r="A10" s="45" t="inlineStr">
+        <is>
+          <t>HU-20</t>
+        </is>
+      </c>
+      <c r="B10" s="46" t="n">
+        <v>5</v>
+      </c>
+      <c r="C10" s="47" t="inlineStr">
+        <is>
+          <t>Reportes</t>
+        </is>
+      </c>
+      <c r="D10" s="47" t="inlineStr">
+        <is>
+          <t>Como gerente de operaciones, quiero exportar la lista de eventos filtrada a CSV, para analizar la informacion en otras herramientas.</t>
+        </is>
+      </c>
+      <c r="E10" s="47" t="inlineStr">
+        <is>
+          <t>1. El boton Exportar respeta los filtros activos.
+2. El archivo incluye todas las columnas del evento y su estado.
+3. La exportacion de hasta 10 000 eventos tarda menos de 10 s.</t>
+        </is>
+      </c>
+      <c r="F10" s="46" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="G10" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" s="47" t="inlineStr">
+        <is>
+          <t>HU-11</t>
+        </is>
+      </c>
+      <c r="I10" s="47" t="inlineStr">
+        <is>
+          <t>HU-11 (S2)</t>
+        </is>
+      </c>
+      <c r="J10" s="47" t="inlineStr">
+        <is>
+          <t>HU-11 (S2)</t>
+        </is>
+      </c>
+      <c r="K10" s="46" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="L10" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="47" t="n"/>
+      <c r="N10" s="47" t="inlineStr">
+        <is>
+          <t>Excluida del conteo del sprint: depende de historias de otro sprint.</t>
+        </is>
+      </c>
+      <c r="O10" s="47" t="inlineStr">
+        <is>
+          <t>Prioridad Could, la menor del backlog. Analisis fuera del sistema.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="15" customHeight="1" s="32">
+      <c r="A11" s="49" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B11" s="50" t="n"/>
+      <c r="C11" s="50" t="n"/>
+      <c r="D11" s="50" t="n"/>
+      <c r="E11" s="50" t="n"/>
+      <c r="F11" s="50" t="n"/>
+      <c r="G11" s="51">
+        <f>SUM(G5:G10)</f>
+        <v/>
+      </c>
+      <c r="H11" s="50" t="n"/>
+      <c r="I11" s="50" t="n"/>
+      <c r="J11" s="50" t="n"/>
+      <c r="K11" s="50" t="n"/>
+      <c r="L11" s="50" t="n"/>
+      <c r="M11" s="50" t="n"/>
+      <c r="N11" s="50" t="n"/>
+      <c r="O11" s="50" t="n"/>
+    </row>
+    <row r="12" s="32"/>
+    <row r="13" s="32"/>
+    <row r="14" s="32"/>
+    <row r="15" s="32"/>
+    <row r="16" s="32"/>
+    <row r="17" s="32"/>
+    <row r="18" s="32"/>
+    <row r="19" s="32"/>
+    <row r="20" s="32"/>
+    <row r="21" s="32"/>
+    <row r="22" s="32"/>
+    <row r="23" s="32"/>
+    <row r="24" s="32"/>
+    <row r="25" s="32"/>
+  </sheetData>
+  <conditionalFormatting sqref="K5:K10">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"NEW"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"PENDING"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+      <formula>"ACTIVE"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
+      <formula>"DONE"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation sqref="K5:K10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"NEW,PENDING,ACTIVE,DONE"</formula1>
+    </dataValidation>
+    <dataValidation sqref="L5:L10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>1</formula2>
+    </dataValidation>
+  </dataValidations>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="42" customWidth="1" style="31" min="1" max="1"/>
@@ -2402,7 +2636,7 @@
     <row r="2" ht="15" customHeight="1" s="32">
       <c r="A2" s="34" t="inlineStr">
         <is>
-          <t>Calculado con formulas sobre la hoja Historias. Cambia un Estado alli y este resumen se actualiza.</t>
+          <t>Calculado con formulas sobre las hojas Historias (MVP) y Backlog. Cambia un Estado alli y este resumen se actualiza.</t>
         </is>
       </c>
     </row>
@@ -2462,31 +2696,31 @@
         </is>
       </c>
       <c r="B6" s="46">
-        <f>COUNTIFS(Historias!$B$5:$B$24,1,Historias!$K$5:$K$24,"NEW")</f>
+        <f>COUNTIFS(Historias!$B$5:$B$18,1,Historias!$K$5:$K$18,"NEW")</f>
         <v/>
       </c>
       <c r="C6" s="46">
-        <f>COUNTIFS(Historias!$B$5:$B$24,1,Historias!$K$5:$K$24,"PENDING")</f>
+        <f>COUNTIFS(Historias!$B$5:$B$18,1,Historias!$K$5:$K$18,"PENDING")</f>
         <v/>
       </c>
       <c r="D6" s="46">
-        <f>COUNTIFS(Historias!$B$5:$B$24,1,Historias!$K$5:$K$24,"ACTIVE")</f>
+        <f>COUNTIFS(Historias!$B$5:$B$18,1,Historias!$K$5:$K$18,"ACTIVE")</f>
         <v/>
       </c>
       <c r="E6" s="46">
-        <f>COUNTIFS(Historias!$B$5:$B$24,1,Historias!$K$5:$K$24,"DONE")</f>
+        <f>COUNTIFS(Historias!$B$5:$B$18,1,Historias!$K$5:$K$18,"DONE")</f>
         <v/>
       </c>
       <c r="F6" s="46">
-        <f>COUNTIFS(Historias!$B$5:$B$24,1)</f>
+        <f>COUNTIFS(Historias!$B$5:$B$18,1)</f>
         <v/>
       </c>
       <c r="G6" s="46">
-        <f>SUMIFS(Historias!$G$5:$G$24,Historias!$B$5:$B$24,1)</f>
+        <f>SUMIFS(Historias!$G$5:$G$18,Historias!$B$5:$B$18,1)</f>
         <v/>
       </c>
       <c r="H6" s="46">
-        <f>SUMIFS(Historias!$G$5:$G$24,Historias!$B$5:$B$24,1)-SUMIFS(Historias!$G$5:$G$24,Historias!$B$5:$B$24,1,Historias!$K$5:$K$24,"PENDING")</f>
+        <f>SUMIFS(Historias!$G$5:$G$18,Historias!$B$5:$B$18,1)-SUMIFS(Historias!$G$5:$G$18,Historias!$B$5:$B$18,1,Historias!$K$5:$K$18,"PENDING")</f>
         <v/>
       </c>
     </row>
@@ -2497,31 +2731,31 @@
         </is>
       </c>
       <c r="B7" s="46">
-        <f>COUNTIFS(Historias!$B$5:$B$24,2,Historias!$K$5:$K$24,"NEW")</f>
+        <f>COUNTIFS(Historias!$B$5:$B$18,2,Historias!$K$5:$K$18,"NEW")</f>
         <v/>
       </c>
       <c r="C7" s="46">
-        <f>COUNTIFS(Historias!$B$5:$B$24,2,Historias!$K$5:$K$24,"PENDING")</f>
+        <f>COUNTIFS(Historias!$B$5:$B$18,2,Historias!$K$5:$K$18,"PENDING")</f>
         <v/>
       </c>
       <c r="D7" s="46">
-        <f>COUNTIFS(Historias!$B$5:$B$24,2,Historias!$K$5:$K$24,"ACTIVE")</f>
+        <f>COUNTIFS(Historias!$B$5:$B$18,2,Historias!$K$5:$K$18,"ACTIVE")</f>
         <v/>
       </c>
       <c r="E7" s="46">
-        <f>COUNTIFS(Historias!$B$5:$B$24,2,Historias!$K$5:$K$24,"DONE")</f>
+        <f>COUNTIFS(Historias!$B$5:$B$18,2,Historias!$K$5:$K$18,"DONE")</f>
         <v/>
       </c>
       <c r="F7" s="46">
-        <f>COUNTIFS(Historias!$B$5:$B$24,2)</f>
+        <f>COUNTIFS(Historias!$B$5:$B$18,2)</f>
         <v/>
       </c>
       <c r="G7" s="46">
-        <f>SUMIFS(Historias!$G$5:$G$24,Historias!$B$5:$B$24,2)</f>
+        <f>SUMIFS(Historias!$G$5:$G$18,Historias!$B$5:$B$18,2)</f>
         <v/>
       </c>
       <c r="H7" s="46">
-        <f>SUMIFS(Historias!$G$5:$G$24,Historias!$B$5:$B$24,2)-SUMIFS(Historias!$G$5:$G$24,Historias!$B$5:$B$24,2,Historias!$K$5:$K$24,"PENDING")</f>
+        <f>SUMIFS(Historias!$G$5:$G$18,Historias!$B$5:$B$18,2)-SUMIFS(Historias!$G$5:$G$18,Historias!$B$5:$B$18,2,Historias!$K$5:$K$18,"PENDING")</f>
         <v/>
       </c>
     </row>
@@ -2532,31 +2766,31 @@
         </is>
       </c>
       <c r="B8" s="46">
-        <f>COUNTIFS(Historias!$B$5:$B$24,3,Historias!$K$5:$K$24,"NEW")</f>
+        <f>COUNTIFS(Historias!$B$5:$B$18,3,Historias!$K$5:$K$18,"NEW")</f>
         <v/>
       </c>
       <c r="C8" s="46">
-        <f>COUNTIFS(Historias!$B$5:$B$24,3,Historias!$K$5:$K$24,"PENDING")</f>
+        <f>COUNTIFS(Historias!$B$5:$B$18,3,Historias!$K$5:$K$18,"PENDING")</f>
         <v/>
       </c>
       <c r="D8" s="46">
-        <f>COUNTIFS(Historias!$B$5:$B$24,3,Historias!$K$5:$K$24,"ACTIVE")</f>
+        <f>COUNTIFS(Historias!$B$5:$B$18,3,Historias!$K$5:$K$18,"ACTIVE")</f>
         <v/>
       </c>
       <c r="E8" s="46">
-        <f>COUNTIFS(Historias!$B$5:$B$24,3,Historias!$K$5:$K$24,"DONE")</f>
+        <f>COUNTIFS(Historias!$B$5:$B$18,3,Historias!$K$5:$K$18,"DONE")</f>
         <v/>
       </c>
       <c r="F8" s="46">
-        <f>COUNTIFS(Historias!$B$5:$B$24,3)</f>
+        <f>COUNTIFS(Historias!$B$5:$B$18,3)</f>
         <v/>
       </c>
       <c r="G8" s="46">
-        <f>SUMIFS(Historias!$G$5:$G$24,Historias!$B$5:$B$24,3)</f>
+        <f>SUMIFS(Historias!$G$5:$G$18,Historias!$B$5:$B$18,3)</f>
         <v/>
       </c>
       <c r="H8" s="46">
-        <f>SUMIFS(Historias!$G$5:$G$24,Historias!$B$5:$B$24,3)-SUMIFS(Historias!$G$5:$G$24,Historias!$B$5:$B$24,3,Historias!$K$5:$K$24,"PENDING")</f>
+        <f>SUMIFS(Historias!$G$5:$G$18,Historias!$B$5:$B$18,3)-SUMIFS(Historias!$G$5:$G$18,Historias!$B$5:$B$18,3,Historias!$K$5:$K$18,"PENDING")</f>
         <v/>
       </c>
     </row>
@@ -2567,31 +2801,31 @@
         </is>
       </c>
       <c r="B9" s="46">
-        <f>COUNTIFS(Historias!$B$5:$B$24,4,Historias!$K$5:$K$24,"NEW")</f>
+        <f>COUNTIFS(Historias!$B$5:$B$18,4,Historias!$K$5:$K$18,"NEW")</f>
         <v/>
       </c>
       <c r="C9" s="46">
-        <f>COUNTIFS(Historias!$B$5:$B$24,4,Historias!$K$5:$K$24,"PENDING")</f>
+        <f>COUNTIFS(Historias!$B$5:$B$18,4,Historias!$K$5:$K$18,"PENDING")</f>
         <v/>
       </c>
       <c r="D9" s="46">
-        <f>COUNTIFS(Historias!$B$5:$B$24,4,Historias!$K$5:$K$24,"ACTIVE")</f>
+        <f>COUNTIFS(Historias!$B$5:$B$18,4,Historias!$K$5:$K$18,"ACTIVE")</f>
         <v/>
       </c>
       <c r="E9" s="46">
-        <f>COUNTIFS(Historias!$B$5:$B$24,4,Historias!$K$5:$K$24,"DONE")</f>
+        <f>COUNTIFS(Historias!$B$5:$B$18,4,Historias!$K$5:$K$18,"DONE")</f>
         <v/>
       </c>
       <c r="F9" s="46">
-        <f>COUNTIFS(Historias!$B$5:$B$24,4)</f>
+        <f>COUNTIFS(Historias!$B$5:$B$18,4)</f>
         <v/>
       </c>
       <c r="G9" s="46">
-        <f>SUMIFS(Historias!$G$5:$G$24,Historias!$B$5:$B$24,4)</f>
+        <f>SUMIFS(Historias!$G$5:$G$18,Historias!$B$5:$B$18,4)</f>
         <v/>
       </c>
       <c r="H9" s="46">
-        <f>SUMIFS(Historias!$G$5:$G$24,Historias!$B$5:$B$24,4)-SUMIFS(Historias!$G$5:$G$24,Historias!$B$5:$B$24,4,Historias!$K$5:$K$24,"PENDING")</f>
+        <f>SUMIFS(Historias!$G$5:$G$18,Historias!$B$5:$B$18,4)-SUMIFS(Historias!$G$5:$G$18,Historias!$B$5:$B$18,4,Historias!$K$5:$K$18,"PENDING")</f>
         <v/>
       </c>
     </row>
@@ -2602,31 +2836,31 @@
         </is>
       </c>
       <c r="B10" s="46">
-        <f>COUNTIFS(Historias!$B$5:$B$24,5,Historias!$K$5:$K$24,"NEW")</f>
+        <f>COUNTIFS(Historias!$B$5:$B$18,5,Historias!$K$5:$K$18,"NEW")</f>
         <v/>
       </c>
       <c r="C10" s="46">
-        <f>COUNTIFS(Historias!$B$5:$B$24,5,Historias!$K$5:$K$24,"PENDING")</f>
+        <f>COUNTIFS(Historias!$B$5:$B$18,5,Historias!$K$5:$K$18,"PENDING")</f>
         <v/>
       </c>
       <c r="D10" s="46">
-        <f>COUNTIFS(Historias!$B$5:$B$24,5,Historias!$K$5:$K$24,"ACTIVE")</f>
+        <f>COUNTIFS(Historias!$B$5:$B$18,5,Historias!$K$5:$K$18,"ACTIVE")</f>
         <v/>
       </c>
       <c r="E10" s="46">
-        <f>COUNTIFS(Historias!$B$5:$B$24,5,Historias!$K$5:$K$24,"DONE")</f>
+        <f>COUNTIFS(Historias!$B$5:$B$18,5,Historias!$K$5:$K$18,"DONE")</f>
         <v/>
       </c>
       <c r="F10" s="46">
-        <f>COUNTIFS(Historias!$B$5:$B$24,5)</f>
+        <f>COUNTIFS(Historias!$B$5:$B$18,5)</f>
         <v/>
       </c>
       <c r="G10" s="46">
-        <f>SUMIFS(Historias!$G$5:$G$24,Historias!$B$5:$B$24,5)</f>
+        <f>SUMIFS(Historias!$G$5:$G$18,Historias!$B$5:$B$18,5)</f>
         <v/>
       </c>
       <c r="H10" s="46">
-        <f>SUMIFS(Historias!$G$5:$G$24,Historias!$B$5:$B$24,5)-SUMIFS(Historias!$G$5:$G$24,Historias!$B$5:$B$24,5,Historias!$K$5:$K$24,"PENDING")</f>
+        <f>SUMIFS(Historias!$G$5:$G$18,Historias!$B$5:$B$18,5)-SUMIFS(Historias!$G$5:$G$18,Historias!$B$5:$B$18,5,Historias!$K$5:$K$18,"PENDING")</f>
         <v/>
       </c>
     </row>
@@ -2690,7 +2924,7 @@
       </c>
       <c r="D14" s="44" t="inlineStr">
         <is>
-          <t>% de los 68 pts</t>
+          <t>% de los 51 pts</t>
         </is>
       </c>
     </row>
@@ -2701,11 +2935,11 @@
         </is>
       </c>
       <c r="B15" s="46">
-        <f>COUNTIF(Historias!$K$5:$K$24,"NEW")</f>
+        <f>COUNTIF(Historias!$K$5:$K$18,"NEW")</f>
         <v/>
       </c>
       <c r="C15" s="46">
-        <f>SUMIF(Historias!$K$5:$K$24,"NEW",Historias!$G$5:$G$24)</f>
+        <f>SUMIF(Historias!$K$5:$K$18,"NEW",Historias!$G$5:$G$18)</f>
         <v/>
       </c>
       <c r="D15" s="54">
@@ -2720,11 +2954,11 @@
         </is>
       </c>
       <c r="B16" s="46">
-        <f>COUNTIF(Historias!$K$5:$K$24,"PENDING")</f>
+        <f>COUNTIF(Historias!$K$5:$K$18,"PENDING")</f>
         <v/>
       </c>
       <c r="C16" s="46">
-        <f>SUMIF(Historias!$K$5:$K$24,"PENDING",Historias!$G$5:$G$24)</f>
+        <f>SUMIF(Historias!$K$5:$K$18,"PENDING",Historias!$G$5:$G$18)</f>
         <v/>
       </c>
       <c r="D16" s="54">
@@ -2739,11 +2973,11 @@
         </is>
       </c>
       <c r="B17" s="46">
-        <f>COUNTIF(Historias!$K$5:$K$24,"ACTIVE")</f>
+        <f>COUNTIF(Historias!$K$5:$K$18,"ACTIVE")</f>
         <v/>
       </c>
       <c r="C17" s="46">
-        <f>SUMIF(Historias!$K$5:$K$24,"ACTIVE",Historias!$G$5:$G$24)</f>
+        <f>SUMIF(Historias!$K$5:$K$18,"ACTIVE",Historias!$G$5:$G$18)</f>
         <v/>
       </c>
       <c r="D17" s="54">
@@ -2758,11 +2992,11 @@
         </is>
       </c>
       <c r="B18" s="46">
-        <f>COUNTIF(Historias!$K$5:$K$24,"DONE")</f>
+        <f>COUNTIF(Historias!$K$5:$K$18,"DONE")</f>
         <v/>
       </c>
       <c r="C18" s="46">
-        <f>SUMIF(Historias!$K$5:$K$24,"DONE",Historias!$G$5:$G$24)</f>
+        <f>SUMIF(Historias!$K$5:$K$18,"DONE",Historias!$G$5:$G$18)</f>
         <v/>
       </c>
       <c r="D18" s="54">
@@ -2781,7 +3015,7 @@
         <v/>
       </c>
       <c r="C19" s="51">
-        <f>SUM(Historias!$G$5:$G$24)</f>
+        <f>SUM(Historias!$G$5:$G$18)</f>
         <v/>
       </c>
       <c r="D19" s="58">
@@ -2803,7 +3037,7 @@
         </is>
       </c>
       <c r="B22" s="60">
-        <f>COUNTIFS(Historias!$B$5:$B$24,1)</f>
+        <f>COUNTIFS(Historias!$B$5:$B$18,1)</f>
         <v/>
       </c>
     </row>
@@ -2814,7 +3048,7 @@
         </is>
       </c>
       <c r="B23" s="60">
-        <f>COUNTIFS(Historias!$B$5:$B$24,1)-COUNTIFS(Historias!$B$5:$B$24,1,Historias!$K$5:$K$24,"PENDING")</f>
+        <f>COUNTIFS(Historias!$B$5:$B$18,1)-COUNTIFS(Historias!$B$5:$B$18,1,Historias!$K$5:$K$18,"PENDING")</f>
         <v/>
       </c>
     </row>
@@ -2825,7 +3059,7 @@
         </is>
       </c>
       <c r="B24" s="60">
-        <f>SUMIFS(Historias!$G$5:$G$24,Historias!$B$5:$B$24,1)</f>
+        <f>SUMIFS(Historias!$G$5:$G$18,Historias!$B$5:$B$18,1)</f>
         <v/>
       </c>
     </row>
@@ -2836,7 +3070,7 @@
         </is>
       </c>
       <c r="B25" s="60">
-        <f>SUMIFS(Historias!$G$5:$G$24,Historias!$B$5:$B$24,1)-SUMIFS(Historias!$G$5:$G$24,Historias!$B$5:$B$24,1,Historias!$K$5:$K$24,"PENDING")</f>
+        <f>SUMIFS(Historias!$G$5:$G$18,Historias!$B$5:$B$18,1)-SUMIFS(Historias!$G$5:$G$18,Historias!$B$5:$B$18,1,Historias!$K$5:$K$18,"PENDING")</f>
         <v/>
       </c>
     </row>
@@ -2847,7 +3081,7 @@
         </is>
       </c>
       <c r="B26" s="60">
-        <f>SUMIFS(Historias!$G$5:$G$24,Historias!$B$5:$B$24,1,Historias!$K$5:$K$24,"PENDING")</f>
+        <f>SUMIFS(Historias!$G$5:$G$18,Historias!$B$5:$B$18,1,Historias!$K$5:$K$18,"PENDING")</f>
         <v/>
       </c>
     </row>
@@ -2874,6 +3108,130 @@
       </c>
       <c r="B28" s="60">
         <f>B27-B25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="35" t="inlineStr">
+        <is>
+          <t>Backlog post-MVP (hoja Backlog)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="44" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B31" s="44" t="inlineStr">
+        <is>
+          <t>Historias</t>
+        </is>
+      </c>
+      <c r="C31" s="44" t="inlineStr">
+        <is>
+          <t>Puntos</t>
+        </is>
+      </c>
+      <c r="D31" s="44" t="inlineStr">
+        <is>
+          <t>% de los 17 pts</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="53" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B32" s="46">
+        <f>COUNTIF(Backlog!$K$5:$K$10,"NEW")</f>
+        <v/>
+      </c>
+      <c r="C32" s="46">
+        <f>SUMIF(Backlog!$K$5:$K$10,"NEW",Backlog!$G$5:$G$10)</f>
+        <v/>
+      </c>
+      <c r="D32" s="54">
+        <f>IFERROR(C32/$C$36,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="55" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="B33" s="46">
+        <f>COUNTIF(Backlog!$K$5:$K$10,"PENDING")</f>
+        <v/>
+      </c>
+      <c r="C33" s="46">
+        <f>SUMIF(Backlog!$K$5:$K$10,"PENDING",Backlog!$G$5:$G$10)</f>
+        <v/>
+      </c>
+      <c r="D33" s="54">
+        <f>IFERROR(C33/$C$36,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="56" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="B34" s="46">
+        <f>COUNTIF(Backlog!$K$5:$K$10,"ACTIVE")</f>
+        <v/>
+      </c>
+      <c r="C34" s="46">
+        <f>SUMIF(Backlog!$K$5:$K$10,"ACTIVE",Backlog!$G$5:$G$10)</f>
+        <v/>
+      </c>
+      <c r="D34" s="54">
+        <f>IFERROR(C34/$C$36,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="57" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="B35" s="46">
+        <f>COUNTIF(Backlog!$K$5:$K$10,"DONE")</f>
+        <v/>
+      </c>
+      <c r="C35" s="46">
+        <f>SUMIF(Backlog!$K$5:$K$10,"DONE",Backlog!$G$5:$G$10)</f>
+        <v/>
+      </c>
+      <c r="D35" s="54">
+        <f>IFERROR(C35/$C$36,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="49" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B36" s="51">
+        <f>SUM(B32:B35)</f>
+        <v/>
+      </c>
+      <c r="C36" s="51">
+        <f>SUM(Backlog!$G$5:$G$10)</f>
+        <v/>
+      </c>
+      <c r="D36" s="58">
+        <f>IFERROR(C36/C36,0)</f>
         <v/>
       </c>
     </row>
@@ -2884,7 +3242,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2913,7 +3271,7 @@
     <row r="2" ht="15" customHeight="1" s="32">
       <c r="A2" s="34" t="inlineStr">
         <is>
-          <t>Alcance evaluado: HU-01, HU-02, HU-04 y HU-15. HU-17 queda fuera por estar en PENDING (depende de HU-03, Sprint 2), por lo que Celery, Redis y Flower salen de la ruta critica del Sprint 1.</t>
+          <t>Alcance evaluado: HU-01, HU-02, HU-04 y HU-14. HU-17 queda fuera por estar en PENDING (depende de HU-03, Sprint 2), por lo que Celery, Redis y Flower salen de la ruta critica del Sprint 1.</t>
         </is>
       </c>
     </row>
@@ -3711,14 +4069,14 @@
       </c>
       <c r="H22" s="47" t="inlineStr">
         <is>
-          <t>No aparece en ninguna parte del documento, pese a que st.dataframe lo requiere y HU-11, HU-14 y HU-20 dependen de el.</t>
+          <t>No aparece en ninguna parte del documento, pese a que st.dataframe lo requiere y HU-11, HU-15 y HU-20 dependen de el.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="45.75" customHeight="1" s="32">
       <c r="A23" s="46" t="inlineStr">
         <is>
-          <t>HU-15</t>
+          <t>HU-14</t>
         </is>
       </c>
       <c r="B23" s="47" t="inlineStr">
@@ -3760,7 +4118,7 @@
     <row r="24" ht="45.75" customHeight="1" s="32">
       <c r="A24" s="46" t="inlineStr">
         <is>
-          <t>HU-15</t>
+          <t>HU-14</t>
         </is>
       </c>
       <c r="B24" s="47" t="inlineStr">
@@ -3802,7 +4160,7 @@
     <row r="25" ht="45.75" customHeight="1" s="32">
       <c r="A25" s="46" t="inlineStr">
         <is>
-          <t>HU-15</t>
+          <t>HU-14</t>
         </is>
       </c>
       <c r="B25" s="47" t="inlineStr">
@@ -3844,7 +4202,7 @@
     <row r="26" ht="45.75" customHeight="1" s="32">
       <c r="A26" s="46" t="inlineStr">
         <is>
-          <t>HU-15</t>
+          <t>HU-14</t>
         </is>
       </c>
       <c r="B26" s="47" t="inlineStr">
@@ -3957,7 +4315,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4099,7 +4457,7 @@
       </c>
       <c r="C8" s="47" t="inlineStr">
         <is>
-          <t>El modelo de datos no contempla la tabla de tokens de acceso a la API, necesaria para HU-15 con autenticacion por token opaco revocable.</t>
+          <t>El modelo de datos no contempla la tabla de tokens de acceso a la API, necesaria para HU-14 con autenticacion por token opaco revocable.</t>
         </is>
       </c>
       <c r="D8" s="47" t="inlineStr">

</xml_diff>